<commit_message>
Update students_latest.xlsx (2026-03-28 02:46:33)
</commit_message>
<xml_diff>
--- a/incoming/students_latest.xlsx
+++ b/incoming/students_latest.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="template" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="students" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43,7 +43,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -51,13 +51,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D9E1F2"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,14 +433,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -441,61 +448,307 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>department</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
           <t>thesis_title</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>manual_research_fields</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>佐藤健</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>社会工学学位プログラム</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>都市交通需要予測に対する時系列深層学習の適用</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>時系列解析;交通工学</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>但木 陸</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>大学入試業務の人員配置最適化における数理モデルの改良</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>田中葵</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>社会工学学位プログラム</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>災害時避難行動データを用いた最適配置モデルの研究</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>防災;最適化</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>吉田 響</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>社会工学・サービス工学学位プログラムにおける修士論文審査員の割り当て問題</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>金原 壮汰</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>LiDARデータに基づく視線および姿勢情報統合による危険行動の動的検出システム〜荷役作業ケース</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>宍戸 唯輝</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>3階層サプライチェーンにおける協調的納期決定アルゴリズム</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>堤 敬信</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>閉鎖型待ち行列ネットワークモデルを用いたシェアサイクルの運用分析</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>寺田 海渡</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>中小企業デフォルト予測における月次流動性預金残高特徴量の有効性検証</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>益子 颯太</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>仕訳データの異常検知モデルの高度化：Data Collaboration解析と摘要欄の活用</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>平井 佑樹</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>仕訳データを用いた利速測定の研究</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>飯田 真実</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>HPVワクチン接種に対する意見の変遷とその要因</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>川井 貫太朗</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>SNSを用いた労働者の集団感情分析</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>冨樫 歩大</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>テキスト情報と財務情報の統合による中小企業の将来性予測</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>出口 達也</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>地域要因を用いた慢性腎臓病患者の悪化予測の研究</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>長谷川 弘貴</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>生体情報とテンソルデータ解析によるコンサート満足度の研究</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>中山 友琉</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>特異値分解を用いた効率的な分散データファインチューニング手法の提案</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>齋藤 彩</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>地域愛着の規定因に関する実証分析：つながりの影響の検討</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>李 宗晟</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>エラスティック光ネットワークにおける通信要求の保持時間を考慮した予約種別リソース割り当て戦略の提案</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>澤口 瑛都</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>列生成法を軸とした電気バスの仕業編成最適化</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>中本 武志</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>大規模言語モデルを活用した非専門家による継続運用可能な勤務表作成手法の検討</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>髙橋 優介</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>重量・近接規制を考慮した異種ドローン経路問題：規制による配送時間・コストへの影響分析</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>鈴木 颯斗</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>最適多分木を用いた解釈可能なクラスタリング</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>佐川 翼</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>社会工学・サービス工学学位プログラムにおける修士論文発表会スケジューリングシステムの開発</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>加田 昌杜</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>学年暦の自動生成 〜曜日変更最小化モデルとその修正の自動化〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>八角 朋樹</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>機械学習モデルと特徴量選択によるファミリーレストラン店舗別売上予測方法の検討</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>山下 穂乃花</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Continual Learning by Null Space of Weight Matrix of Previous Task for Deep Neural Network</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>崔 涵喬</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>観光客のセグメンテーションとマーケティングへの応用可能性に関する研究</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update students_latest.xlsx (2026-03-28 02:55:08)
</commit_message>
<xml_diff>
--- a/incoming/students_latest.xlsx
+++ b/incoming/students_latest.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="students" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="teachers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,322 +433,212 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>student_name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>thesis_title</t>
+          <t>teacher_name</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>但木 陸</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>大学入試業務の人員配置最適化における数理モデルの改良</t>
+          <t>吉瀬章子</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>吉田 響</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>社会工学・サービス工学学位プログラムにおける修士論文審査員の割り当て問題</t>
+          <t>小西葉子</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>金原 壮汰</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>LiDARデータに基づく視線および姿勢情報統合による危険行動の動的検出システム〜荷役作業ケース</t>
+          <t>高野祐一</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>宍戸 唯輝</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>3階層サプライチェーンにおける協調的納期決定アルゴリズム</t>
+          <t>繆瑩</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>堤 敬信</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>閉鎖型待ち行列ネットワークモデルを用いたシェアサイクルの運用分析</t>
+          <t>有馬澄佳</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>寺田 海渡</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>中小企業デフォルト予測における月次流動性預金残高特徴量の有効性検証</t>
+          <t>イリチュ美佳</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>益子 颯太</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>仕訳データの異常検知モデルの高度化：Data Collaboration解析と摘要欄の活用</t>
+          <t>志田洋平</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>平井 佑樹</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>仕訳データを用いた利速測定の研究</t>
+          <t>大久保正勝</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>飯田 真実</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>HPVワクチン接種に対する意見の変遷とその要因</t>
+          <t>Phung-DucTuan</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>川井 貫太朗</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>SNSを用いた労働者の集団感情分析</t>
+          <t>張勇兵</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>冨樫 歩大</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>テキスト情報と財務情報の統合による中小企業の将来性予測</t>
+          <t>岡田幸彦</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>出口 達也</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>地域要因を用いた慢性腎臓病患者の悪化予測の研究</t>
+          <t>上市秀雄</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>長谷川 弘貴</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>生体情報とテンソルデータ解析によるコンサート満足度の研究</t>
+          <t>黒瀬雄大</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>中山 友琉</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>特異値分解を用いた効率的な分散データファインチューニング手法の提案</t>
+          <t>佐野幸恵</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>齋藤 彩</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>地域愛着の規定因に関する実証分析：つながりの影響の検討</t>
+          <t>秋山英三</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>李 宗晟</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>エラスティック光ネットワークにおける通信要求の保持時間を考慮した予約種別リソース割り当て戦略の提案</t>
+          <t>TranLamAnhDuong</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>澤口 瑛都</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>列生成法を軸とした電気バスの仕業編成最適化</t>
+          <t>LiuTianxiang</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>中本 武志</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>大規模言語モデルを活用した非専門家による継続運用可能な勤務表作成手法の検討</t>
+          <t>奥島真一郎</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>髙橋 優介</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>重量・近接規制を考慮した異種ドローン経路問題：規制による配送時間・コストへの影響分析</t>
+          <t>八森正泰</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>鈴木 颯斗</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>最適多分木を用いた解釈可能なクラスタリング</t>
+          <t>原田信行</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>佐川 翼</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>社会工学・サービス工学学位プログラムにおける修士論文発表会スケジューリングシステムの開発</t>
+          <t>藤井さやか</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>加田 昌杜</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>学年暦の自動生成 〜曜日変更最小化モデルとその修正の自動化〜</t>
+          <t>繁野麻衣子</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>八角 朋樹</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>機械学習モデルと特徴量選択によるファミリーレストラン店舗別売上予測方法の検討</t>
+          <t>木下陽平</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>山下 穂乃花</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Continual Learning by Null Space of Weight Matrix of Previous Task for Deep Neural Network</t>
+          <t>讃井知</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>崔 涵喬</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>観光客のセグメンテーションとマーケティングへの応用可能性に関する研究</t>
+          <t>作道真理</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>髙橋裕紀</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>大西正輝</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>岡本直久</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: pending student excel
</commit_message>
<xml_diff>
--- a/incoming/students_latest.xlsx
+++ b/incoming/students_latest.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="teachers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="students" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,212 +433,322 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>teacher_name</t>
+          <t>student_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>thesis_title</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>吉瀬章子</t>
+          <t>但木 陸</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>大学入試業務の人員配置最適化における数理モデルの改良</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>小西葉子</t>
+          <t>吉田 響</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>社会工学・サービス工学学位プログラムにおける修士論文審査員の割り当て問題</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>高野祐一</t>
+          <t>金原 壮汰</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>LiDARデータに基づく視線および姿勢情報統合による危険行動の動的検出システム〜荷役作業ケース</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>繆瑩</t>
+          <t>宍戸 唯輝</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>3階層サプライチェーンにおける協調的納期決定アルゴリズム</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>有馬澄佳</t>
+          <t>堤 敬信</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>閉鎖型待ち行列ネットワークモデルを用いたシェアサイクルの運用分析</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>イリチュ美佳</t>
+          <t>寺田 海渡</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>中小企業デフォルト予測における月次流動性預金残高特徴量の有効性検証</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>志田洋平</t>
+          <t>益子 颯太</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>仕訳データの異常検知モデルの高度化：Data Collaboration解析と摘要欄の活用</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>大久保正勝</t>
+          <t>平井 佑樹</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>仕訳データを用いた利速測定の研究</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Phung-DucTuan</t>
+          <t>飯田 真実</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>HPVワクチン接種に対する意見の変遷とその要因</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>張勇兵</t>
+          <t>川井 貫太朗</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>SNSを用いた労働者の集団感情分析</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>岡田幸彦</t>
+          <t>冨樫 歩大</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>テキスト情報と財務情報の統合による中小企業の将来性予測</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>上市秀雄</t>
+          <t>出口 達也</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>地域要因を用いた慢性腎臓病患者の悪化予測の研究</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>黒瀬雄大</t>
+          <t>長谷川 弘貴</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>生体情報とテンソルデータ解析によるコンサート満足度の研究</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>佐野幸恵</t>
+          <t>中山 友琉</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>特異値分解を用いた効率的な分散データファインチューニング手法の提案</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>秋山英三</t>
+          <t>齋藤 彩</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>地域愛着の規定因に関する実証分析：つながりの影響の検討</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TranLamAnhDuong</t>
+          <t>李 宗晟</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>エラスティック光ネットワークにおける通信要求の保持時間を考慮した予約種別リソース割り当て戦略の提案</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>LiuTianxiang</t>
+          <t>澤口 瑛都</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>列生成法を軸とした電気バスの仕業編成最適化</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>奥島真一郎</t>
+          <t>中本 武志</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>大規模言語モデルを活用した非専門家による継続運用可能な勤務表作成手法の検討</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>八森正泰</t>
+          <t>髙橋 優介</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>重量・近接規制を考慮した異種ドローン経路問題：規制による配送時間・コストへの影響分析</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>原田信行</t>
+          <t>鈴木 颯斗</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>最適多分木を用いた解釈可能なクラスタリング</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>藤井さやか</t>
+          <t>佐川 翼</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>社会工学・サービス工学学位プログラムにおける修士論文発表会スケジューリングシステムの開発</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>繁野麻衣子</t>
+          <t>加田 昌杜</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>学年暦の自動生成 〜曜日変更最小化モデルとその修正の自動化〜</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>木下陽平</t>
+          <t>八角 朋樹</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>機械学習モデルと特徴量選択によるファミリーレストラン店舗別売上予測方法の検討</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>讃井知</t>
+          <t>山下 穂乃花</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Continual Learning by Null Space of Weight Matrix of Previous Task for Deep Neural Network</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>作道真理</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>髙橋裕紀</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>大西正輝</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>岡本直久</t>
+          <t>崔 涵喬</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>観光客のセグメンテーションとマーケティングへの応用可能性に関する研究</t>
         </is>
       </c>
     </row>

</xml_diff>